<commit_message>
PA quote E2E developed
</commit_message>
<xml_diff>
--- a/pages/UATStability.xlsx
+++ b/pages/UATStability.xlsx
@@ -8,19 +8,30 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E275B8-A85C-4DFB-9A40-613603FC57C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DCA5435-2E9C-4EDF-84F8-B1C14B2AF81E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t>S.No</t>
   </si>
@@ -53,6 +64,9 @@
   </si>
   <si>
     <t>1000062674</t>
+  </si>
+  <si>
+    <t>PA</t>
   </si>
 </sst>
 </file>
@@ -123,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -143,11 +157,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -463,17 +480,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" style="4" customWidth="1"/>
     <col min="2" max="2" width="14" style="4" customWidth="1"/>
-    <col min="3" max="7" width="15" style="4" customWidth="1"/>
+    <col min="3" max="6" width="15" style="4" customWidth="1"/>
+    <col min="7" max="7" width="21.08984375" style="4" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="10" max="10" width="12.453125" customWidth="1"/>
+    <col min="11" max="11" width="13.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" s="1" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -496,8 +515,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="8">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="7">
         <v>1</v>
       </c>
       <c r="B2" s="6"/>
@@ -511,8 +530,8 @@
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="8">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="7">
         <v>2</v>
       </c>
       <c r="B3" s="6"/>
@@ -526,8 +545,8 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="8">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="7">
         <v>3</v>
       </c>
       <c r="B4" s="6"/>
@@ -538,23 +557,33 @@
       <c r="E4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="7"/>
+      <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="J4" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="8"/>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="7">
+        <v>4</v>
+      </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6" t="s">
+        <v>11</v>
+      </c>
       <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="J5" s="8">
+        <v>1000063122</v>
+      </c>
+      <c r="K5" s="9">
+        <v>402000066256</v>
+      </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="8"/>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
@@ -565,5 +594,8 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
+  <ignoredErrors>
+    <ignoredError sqref="J4" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
UAt stability Excel sheet updated
</commit_message>
<xml_diff>
--- a/pages/UATStability.xlsx
+++ b/pages/UATStability.xlsx
@@ -1,47 +1,111 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3935BBC7-8F64-45A4-AE56-26AB7CE56F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+  <si>
+    <t>S.No</t>
+  </si>
+  <si>
+    <t>Automation/Manual</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Motor Type</t>
+  </si>
+  <si>
+    <t>Quote Number</t>
+  </si>
+  <si>
+    <t>Policy Number</t>
+  </si>
+  <si>
+    <t>MC</t>
+  </si>
+  <si>
+    <t>Comprehensive</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>CV</t>
+  </si>
+  <si>
+    <t>1000062674</t>
+  </si>
+  <si>
+    <t>PA</t>
+  </si>
+  <si>
+    <t>1000063210</t>
+  </si>
+  <si>
+    <t>00000402000066330</t>
+  </si>
+  <si>
+    <t>1000063212</t>
+  </si>
+  <si>
+    <t>00000402000066332</t>
+  </si>
+  <si>
+    <t>1000063131</t>
+  </si>
+  <si>
+    <t>1000063183</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="12"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -80,105 +144,52 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -478,170 +489,152 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col width="15" customWidth="1" style="4" min="1" max="1"/>
-    <col width="14" customWidth="1" style="4" min="2" max="2"/>
-    <col width="15" customWidth="1" style="4" min="3" max="6"/>
-    <col width="21.08984375" customWidth="1" style="4" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="12.453125" customWidth="1" min="10" max="10"/>
-    <col width="13.26953125" customWidth="1" min="11" max="11"/>
+    <col min="1" max="1" width="15" style="4" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
+    <col min="3" max="6" width="15" style="4" customWidth="1"/>
+    <col min="7" max="7" width="21.08984375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="10" max="10" width="12.453125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="19.6328125" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31" customFormat="1" customHeight="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>S.No</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Automation/Manual</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Motor Type</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Quote Number</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Policy Number</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="n">
+    <row r="1" spans="1:11" s="1" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="n"/>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Comprehensive</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="n">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>Comprehensive</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="n">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Comprehensive</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>1000062674</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="E1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>1000063183</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>00000402000066301</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="n">
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A3" s="7">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="J4" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="7">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="F5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="9">
         <v>1000063122</v>
       </c>
-      <c r="K5" s="8" t="n">
+      <c r="K5" s="10">
         <v>402000066256</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>1000063131</t>
-        </is>
-      </c>
-      <c r="K6" s="8" t="n">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="10">
         <v>402000066265</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K7" s="10">
+        <v>402000066301</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated the folder and codecls
</commit_message>
<xml_diff>
--- a/pages/UATStability.xlsx
+++ b/pages/UATStability.xlsx
@@ -968,11 +968,27 @@
       <c r="A10" s="7" t="n"/>
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
       <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>1000063666</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>00000402000066661</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>24-03-2026</t>
+        </is>
+      </c>
       <c r="I10" s="12" t="n"/>
       <c r="J10" s="12" t="n"/>
     </row>
@@ -980,11 +996,27 @@
       <c r="A11" s="7" t="n"/>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>1000064068</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>00000402000067037</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>30-03-2026</t>
+        </is>
+      </c>
       <c r="I11" s="12" t="n"/>
       <c r="J11" s="12" t="n"/>
     </row>

</xml_diff>

<commit_message>
CV & PC updated
</commit_message>
<xml_diff>
--- a/pages/UATStability.xlsx
+++ b/pages/UATStability.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F14A70F-7068-4646-83BA-5CFD86F19133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA74C06-8978-4CD9-AC42-022B588A9806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
   <si>
     <t>S.No</t>
   </si>
@@ -64,6 +64,9 @@
     <t>PA</t>
   </si>
   <si>
+    <t>Personal Accident Safe</t>
+  </si>
+  <si>
     <t>1000067625</t>
   </si>
   <si>
@@ -77,7 +80,19 @@
 Validated Manually</t>
   </si>
   <si>
-    <t>Personal Accident Safe</t>
+    <t>RV</t>
+  </si>
+  <si>
+    <t>CV</t>
+  </si>
+  <si>
+    <t>TP, Fire &amp; Theft</t>
+  </si>
+  <si>
+    <t>1000067677</t>
+  </si>
+  <si>
+    <t>00000402000069730</t>
   </si>
 </sst>
 </file>
@@ -569,35 +584,55 @@
         <v>12</v>
       </c>
       <c r="E2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>13</v>
+      <c r="J2" s="9" t="s">
+        <v>17</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>14</v>
+    </row>
+    <row r="3" spans="1:10" ht="28" x14ac:dyDescent="0.35">
+      <c r="A3" s="7">
+        <v>2</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>15</v>
+      <c r="B3" s="10" t="s">
+        <v>10</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="C3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="9" t="s">
-        <v>16</v>
+      <c r="I3" s="9" t="s">
+        <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="7"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
+      <c r="J3" s="9" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="7"/>

</xml_diff>

<commit_message>
Added Endorsement and custom command
</commit_message>
<xml_diff>
--- a/pages/UATStability.xlsx
+++ b/pages/UATStability.xlsx
@@ -211,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -246,10 +246,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1412,8 +1408,8 @@
       <c r="F61" s="5"/>
       <c r="G61" s="5"/>
       <c r="H61" s="5"/>
-      <c r="I61" s="15"/>
-      <c r="J61" s="15"/>
+      <c r="I61" s="13"/>
+      <c r="J61" s="13"/>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="5"/>
@@ -1424,8 +1420,8 @@
       <c r="F62" s="5"/>
       <c r="G62" s="5"/>
       <c r="H62" s="5"/>
-      <c r="I62" s="15"/>
-      <c r="J62" s="15"/>
+      <c r="I62" s="13"/>
+      <c r="J62" s="13"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="5"/>
@@ -1436,8 +1432,8 @@
       <c r="F63" s="5"/>
       <c r="G63" s="5"/>
       <c r="H63" s="5"/>
-      <c r="I63" s="15"/>
-      <c r="J63" s="15"/>
+      <c r="I63" s="13"/>
+      <c r="J63" s="13"/>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" s="5"/>
@@ -1448,8 +1444,8 @@
       <c r="F64" s="5"/>
       <c r="G64" s="5"/>
       <c r="H64" s="5"/>
-      <c r="I64" s="15"/>
-      <c r="J64" s="15"/>
+      <c r="I64" s="13"/>
+      <c r="J64" s="13"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="5"/>
@@ -1460,8 +1456,8 @@
       <c r="F65" s="5"/>
       <c r="G65" s="5"/>
       <c r="H65" s="5"/>
-      <c r="I65" s="15"/>
-      <c r="J65" s="15"/>
+      <c r="I65" s="13"/>
+      <c r="J65" s="13"/>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" s="5"/>
@@ -1472,8 +1468,8 @@
       <c r="F66" s="5"/>
       <c r="G66" s="5"/>
       <c r="H66" s="5"/>
-      <c r="I66" s="15"/>
-      <c r="J66" s="15"/>
+      <c r="I66" s="13"/>
+      <c r="J66" s="13"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" s="5"/>
@@ -1484,8 +1480,8 @@
       <c r="F67" s="5"/>
       <c r="G67" s="5"/>
       <c r="H67" s="5"/>
-      <c r="I67" s="15"/>
-      <c r="J67" s="15"/>
+      <c r="I67" s="13"/>
+      <c r="J67" s="13"/>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="5"/>
@@ -1496,8 +1492,8 @@
       <c r="F68" s="5"/>
       <c r="G68" s="5"/>
       <c r="H68" s="5"/>
-      <c r="I68" s="15"/>
-      <c r="J68" s="15"/>
+      <c r="I68" s="13"/>
+      <c r="J68" s="13"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="5"/>
@@ -1508,8 +1504,8 @@
       <c r="F69" s="5"/>
       <c r="G69" s="5"/>
       <c r="H69" s="5"/>
-      <c r="I69" s="15"/>
-      <c r="J69" s="15"/>
+      <c r="I69" s="13"/>
+      <c r="J69" s="13"/>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" s="5"/>
@@ -1520,8 +1516,8 @@
       <c r="F70" s="5"/>
       <c r="G70" s="5"/>
       <c r="H70" s="5"/>
-      <c r="I70" s="15"/>
-      <c r="J70" s="15"/>
+      <c r="I70" s="13"/>
+      <c r="J70" s="13"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" s="5"/>
@@ -1532,8 +1528,8 @@
       <c r="F71" s="5"/>
       <c r="G71" s="5"/>
       <c r="H71" s="5"/>
-      <c r="I71" s="15"/>
-      <c r="J71" s="15"/>
+      <c r="I71" s="13"/>
+      <c r="J71" s="13"/>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="5"/>
@@ -1544,8 +1540,8 @@
       <c r="F72" s="5"/>
       <c r="G72" s="5"/>
       <c r="H72" s="5"/>
-      <c r="I72" s="15"/>
-      <c r="J72" s="15"/>
+      <c r="I72" s="13"/>
+      <c r="J72" s="13"/>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="5"/>
@@ -1556,8 +1552,8 @@
       <c r="F73" s="5"/>
       <c r="G73" s="5"/>
       <c r="H73" s="5"/>
-      <c r="I73" s="15"/>
-      <c r="J73" s="15"/>
+      <c r="I73" s="13"/>
+      <c r="J73" s="13"/>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" s="5"/>
@@ -1568,8 +1564,8 @@
       <c r="F74" s="5"/>
       <c r="G74" s="5"/>
       <c r="H74" s="5"/>
-      <c r="I74" s="15"/>
-      <c r="J74" s="15"/>
+      <c r="I74" s="13"/>
+      <c r="J74" s="13"/>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" s="5"/>
@@ -1580,8 +1576,8 @@
       <c r="F75" s="5"/>
       <c r="G75" s="5"/>
       <c r="H75" s="5"/>
-      <c r="I75" s="15"/>
-      <c r="J75" s="15"/>
+      <c r="I75" s="13"/>
+      <c r="J75" s="13"/>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76" s="5"/>
@@ -1592,8 +1588,8 @@
       <c r="F76" s="5"/>
       <c r="G76" s="5"/>
       <c r="H76" s="5"/>
-      <c r="I76" s="15"/>
-      <c r="J76" s="15"/>
+      <c r="I76" s="13"/>
+      <c r="J76" s="13"/>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" s="5"/>
@@ -1604,8 +1600,8 @@
       <c r="F77" s="5"/>
       <c r="G77" s="5"/>
       <c r="H77" s="5"/>
-      <c r="I77" s="15"/>
-      <c r="J77" s="15"/>
+      <c r="I77" s="13"/>
+      <c r="J77" s="13"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="5"/>
@@ -1616,8 +1612,8 @@
       <c r="F78" s="5"/>
       <c r="G78" s="5"/>
       <c r="H78" s="5"/>
-      <c r="I78" s="15"/>
-      <c r="J78" s="15"/>
+      <c r="I78" s="13"/>
+      <c r="J78" s="13"/>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A79" s="5"/>
@@ -1628,8 +1624,8 @@
       <c r="F79" s="5"/>
       <c r="G79" s="5"/>
       <c r="H79" s="5"/>
-      <c r="I79" s="15"/>
-      <c r="J79" s="15"/>
+      <c r="I79" s="13"/>
+      <c r="J79" s="13"/>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" s="5"/>
@@ -1640,8 +1636,8 @@
       <c r="F80" s="5"/>
       <c r="G80" s="5"/>
       <c r="H80" s="5"/>
-      <c r="I80" s="15"/>
-      <c r="J80" s="15"/>
+      <c r="I80" s="13"/>
+      <c r="J80" s="13"/>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A81" s="5"/>
@@ -1652,8 +1648,8 @@
       <c r="F81" s="5"/>
       <c r="G81" s="5"/>
       <c r="H81" s="5"/>
-      <c r="I81" s="15"/>
-      <c r="J81" s="15"/>
+      <c r="I81" s="13"/>
+      <c r="J81" s="13"/>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A82" s="5"/>
@@ -1664,8 +1660,8 @@
       <c r="F82" s="5"/>
       <c r="G82" s="5"/>
       <c r="H82" s="5"/>
-      <c r="I82" s="15"/>
-      <c r="J82" s="15"/>
+      <c r="I82" s="13"/>
+      <c r="J82" s="13"/>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A83" s="5"/>
@@ -1676,8 +1672,8 @@
       <c r="F83" s="5"/>
       <c r="G83" s="5"/>
       <c r="H83" s="5"/>
-      <c r="I83" s="15"/>
-      <c r="J83" s="15"/>
+      <c r="I83" s="13"/>
+      <c r="J83" s="13"/>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" s="5"/>
@@ -1688,8 +1684,8 @@
       <c r="F84" s="5"/>
       <c r="G84" s="5"/>
       <c r="H84" s="5"/>
-      <c r="I84" s="15"/>
-      <c r="J84" s="15"/>
+      <c r="I84" s="13"/>
+      <c r="J84" s="13"/>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A85" s="5"/>
@@ -1700,8 +1696,8 @@
       <c r="F85" s="5"/>
       <c r="G85" s="5"/>
       <c r="H85" s="5"/>
-      <c r="I85" s="15"/>
-      <c r="J85" s="15"/>
+      <c r="I85" s="13"/>
+      <c r="J85" s="13"/>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" s="5"/>
@@ -1712,8 +1708,8 @@
       <c r="F86" s="5"/>
       <c r="G86" s="5"/>
       <c r="H86" s="5"/>
-      <c r="I86" s="15"/>
-      <c r="J86" s="15"/>
+      <c r="I86" s="13"/>
+      <c r="J86" s="13"/>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" s="5"/>
@@ -1724,8 +1720,8 @@
       <c r="F87" s="5"/>
       <c r="G87" s="5"/>
       <c r="H87" s="5"/>
-      <c r="I87" s="15"/>
-      <c r="J87" s="15"/>
+      <c r="I87" s="13"/>
+      <c r="J87" s="13"/>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A88" s="5"/>
@@ -1736,8 +1732,8 @@
       <c r="F88" s="5"/>
       <c r="G88" s="5"/>
       <c r="H88" s="5"/>
-      <c r="I88" s="15"/>
-      <c r="J88" s="15"/>
+      <c r="I88" s="13"/>
+      <c r="J88" s="13"/>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" s="5"/>
@@ -1748,8 +1744,8 @@
       <c r="F89" s="5"/>
       <c r="G89" s="5"/>
       <c r="H89" s="5"/>
-      <c r="I89" s="15"/>
-      <c r="J89" s="15"/>
+      <c r="I89" s="13"/>
+      <c r="J89" s="13"/>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A90" s="5"/>
@@ -1760,8 +1756,8 @@
       <c r="F90" s="5"/>
       <c r="G90" s="5"/>
       <c r="H90" s="5"/>
-      <c r="I90" s="15"/>
-      <c r="J90" s="15"/>
+      <c r="I90" s="13"/>
+      <c r="J90" s="13"/>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A91" s="5"/>
@@ -1772,8 +1768,8 @@
       <c r="F91" s="5"/>
       <c r="G91" s="5"/>
       <c r="H91" s="5"/>
-      <c r="I91" s="15"/>
-      <c r="J91" s="15"/>
+      <c r="I91" s="13"/>
+      <c r="J91" s="13"/>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A92" s="5"/>
@@ -1784,8 +1780,8 @@
       <c r="F92" s="5"/>
       <c r="G92" s="5"/>
       <c r="H92" s="5"/>
-      <c r="I92" s="15"/>
-      <c r="J92" s="15"/>
+      <c r="I92" s="13"/>
+      <c r="J92" s="13"/>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A93" s="5"/>
@@ -1796,8 +1792,8 @@
       <c r="F93" s="5"/>
       <c r="G93" s="5"/>
       <c r="H93" s="5"/>
-      <c r="I93" s="15"/>
-      <c r="J93" s="15"/>
+      <c r="I93" s="13"/>
+      <c r="J93" s="13"/>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" s="5"/>
@@ -1808,8 +1804,8 @@
       <c r="F94" s="5"/>
       <c r="G94" s="5"/>
       <c r="H94" s="5"/>
-      <c r="I94" s="15"/>
-      <c r="J94" s="15"/>
+      <c r="I94" s="13"/>
+      <c r="J94" s="13"/>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" s="5"/>
@@ -1820,8 +1816,8 @@
       <c r="F95" s="5"/>
       <c r="G95" s="5"/>
       <c r="H95" s="5"/>
-      <c r="I95" s="15"/>
-      <c r="J95" s="15"/>
+      <c r="I95" s="13"/>
+      <c r="J95" s="13"/>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" s="5"/>
@@ -1832,8 +1828,8 @@
       <c r="F96" s="5"/>
       <c r="G96" s="5"/>
       <c r="H96" s="5"/>
-      <c r="I96" s="15"/>
-      <c r="J96" s="15"/>
+      <c r="I96" s="13"/>
+      <c r="J96" s="13"/>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" s="5"/>
@@ -1844,8 +1840,8 @@
       <c r="F97" s="5"/>
       <c r="G97" s="5"/>
       <c r="H97" s="5"/>
-      <c r="I97" s="15"/>
-      <c r="J97" s="15"/>
+      <c r="I97" s="13"/>
+      <c r="J97" s="13"/>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" s="5"/>
@@ -1856,8 +1852,8 @@
       <c r="F98" s="5"/>
       <c r="G98" s="5"/>
       <c r="H98" s="5"/>
-      <c r="I98" s="15"/>
-      <c r="J98" s="15"/>
+      <c r="I98" s="13"/>
+      <c r="J98" s="13"/>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" s="5"/>
@@ -1868,8 +1864,8 @@
       <c r="F99" s="5"/>
       <c r="G99" s="5"/>
       <c r="H99" s="5"/>
-      <c r="I99" s="15"/>
-      <c r="J99" s="15"/>
+      <c r="I99" s="13"/>
+      <c r="J99" s="13"/>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" s="5"/>
@@ -1880,8 +1876,8 @@
       <c r="F100" s="5"/>
       <c r="G100" s="5"/>
       <c r="H100" s="5"/>
-      <c r="I100" s="15"/>
-      <c r="J100" s="15"/>
+      <c r="I100" s="13"/>
+      <c r="J100" s="13"/>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" s="5"/>
@@ -1892,8 +1888,8 @@
       <c r="F101" s="5"/>
       <c r="G101" s="5"/>
       <c r="H101" s="5"/>
-      <c r="I101" s="15"/>
-      <c r="J101" s="15"/>
+      <c r="I101" s="13"/>
+      <c r="J101" s="13"/>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" s="5"/>
@@ -1904,8 +1900,8 @@
       <c r="F102" s="5"/>
       <c r="G102" s="5"/>
       <c r="H102" s="5"/>
-      <c r="I102" s="15"/>
-      <c r="J102" s="15"/>
+      <c r="I102" s="13"/>
+      <c r="J102" s="13"/>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" s="5"/>
@@ -1916,8 +1912,8 @@
       <c r="F103" s="5"/>
       <c r="G103" s="5"/>
       <c r="H103" s="5"/>
-      <c r="I103" s="15"/>
-      <c r="J103" s="15"/>
+      <c r="I103" s="13"/>
+      <c r="J103" s="13"/>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" s="5"/>
@@ -1928,8 +1924,8 @@
       <c r="F104" s="5"/>
       <c r="G104" s="5"/>
       <c r="H104" s="5"/>
-      <c r="I104" s="15"/>
-      <c r="J104" s="15"/>
+      <c r="I104" s="13"/>
+      <c r="J104" s="13"/>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" s="5"/>
@@ -1940,8 +1936,8 @@
       <c r="F105" s="5"/>
       <c r="G105" s="5"/>
       <c r="H105" s="5"/>
-      <c r="I105" s="15"/>
-      <c r="J105" s="15"/>
+      <c r="I105" s="13"/>
+      <c r="J105" s="13"/>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" s="5"/>
@@ -1952,8 +1948,8 @@
       <c r="F106" s="5"/>
       <c r="G106" s="5"/>
       <c r="H106" s="5"/>
-      <c r="I106" s="15"/>
-      <c r="J106" s="15"/>
+      <c r="I106" s="13"/>
+      <c r="J106" s="13"/>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" s="5"/>
@@ -1964,8 +1960,8 @@
       <c r="F107" s="5"/>
       <c r="G107" s="5"/>
       <c r="H107" s="5"/>
-      <c r="I107" s="15"/>
-      <c r="J107" s="15"/>
+      <c r="I107" s="13"/>
+      <c r="J107" s="13"/>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" s="5"/>
@@ -1976,8 +1972,8 @@
       <c r="F108" s="5"/>
       <c r="G108" s="5"/>
       <c r="H108" s="5"/>
-      <c r="I108" s="15"/>
-      <c r="J108" s="15"/>
+      <c r="I108" s="13"/>
+      <c r="J108" s="13"/>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="5"/>
@@ -1988,8 +1984,8 @@
       <c r="F109" s="5"/>
       <c r="G109" s="5"/>
       <c r="H109" s="5"/>
-      <c r="I109" s="15"/>
-      <c r="J109" s="15"/>
+      <c r="I109" s="13"/>
+      <c r="J109" s="13"/>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="5"/>
@@ -2000,8 +1996,8 @@
       <c r="F110" s="5"/>
       <c r="G110" s="5"/>
       <c r="H110" s="5"/>
-      <c r="I110" s="15"/>
-      <c r="J110" s="15"/>
+      <c r="I110" s="13"/>
+      <c r="J110" s="13"/>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="5"/>
@@ -2012,8 +2008,8 @@
       <c r="F111" s="5"/>
       <c r="G111" s="5"/>
       <c r="H111" s="5"/>
-      <c r="I111" s="15"/>
-      <c r="J111" s="15"/>
+      <c r="I111" s="13"/>
+      <c r="J111" s="13"/>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="5"/>
@@ -2024,8 +2020,8 @@
       <c r="F112" s="5"/>
       <c r="G112" s="5"/>
       <c r="H112" s="5"/>
-      <c r="I112" s="15"/>
-      <c r="J112" s="15"/>
+      <c r="I112" s="13"/>
+      <c r="J112" s="13"/>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A113" s="5"/>
@@ -2036,8 +2032,8 @@
       <c r="F113" s="5"/>
       <c r="G113" s="5"/>
       <c r="H113" s="5"/>
-      <c r="I113" s="15"/>
-      <c r="J113" s="15"/>
+      <c r="I113" s="13"/>
+      <c r="J113" s="13"/>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A114" s="5"/>
@@ -2048,8 +2044,8 @@
       <c r="F114" s="5"/>
       <c r="G114" s="5"/>
       <c r="H114" s="5"/>
-      <c r="I114" s="15"/>
-      <c r="J114" s="15"/>
+      <c r="I114" s="13"/>
+      <c r="J114" s="13"/>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A115" s="5"/>
@@ -2060,8 +2056,8 @@
       <c r="F115" s="5"/>
       <c r="G115" s="5"/>
       <c r="H115" s="5"/>
-      <c r="I115" s="15"/>
-      <c r="J115" s="15"/>
+      <c r="I115" s="13"/>
+      <c r="J115" s="13"/>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A116" s="5"/>
@@ -2072,8 +2068,8 @@
       <c r="F116" s="5"/>
       <c r="G116" s="5"/>
       <c r="H116" s="5"/>
-      <c r="I116" s="15"/>
-      <c r="J116" s="15"/>
+      <c r="I116" s="13"/>
+      <c r="J116" s="13"/>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A117" s="5"/>
@@ -2084,8 +2080,8 @@
       <c r="F117" s="5"/>
       <c r="G117" s="5"/>
       <c r="H117" s="5"/>
-      <c r="I117" s="15"/>
-      <c r="J117" s="15"/>
+      <c r="I117" s="13"/>
+      <c r="J117" s="13"/>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" s="5"/>
@@ -2096,8 +2092,8 @@
       <c r="F118" s="5"/>
       <c r="G118" s="5"/>
       <c r="H118" s="5"/>
-      <c r="I118" s="15"/>
-      <c r="J118" s="15"/>
+      <c r="I118" s="13"/>
+      <c r="J118" s="13"/>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A119" s="5"/>
@@ -2108,8 +2104,8 @@
       <c r="F119" s="5"/>
       <c r="G119" s="5"/>
       <c r="H119" s="5"/>
-      <c r="I119" s="15"/>
-      <c r="J119" s="15"/>
+      <c r="I119" s="13"/>
+      <c r="J119" s="13"/>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" s="5"/>
@@ -2120,8 +2116,8 @@
       <c r="F120" s="5"/>
       <c r="G120" s="5"/>
       <c r="H120" s="5"/>
-      <c r="I120" s="15"/>
-      <c r="J120" s="15"/>
+      <c r="I120" s="13"/>
+      <c r="J120" s="13"/>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A121" s="5"/>
@@ -2132,8 +2128,8 @@
       <c r="F121" s="5"/>
       <c r="G121" s="5"/>
       <c r="H121" s="5"/>
-      <c r="I121" s="15"/>
-      <c r="J121" s="15"/>
+      <c r="I121" s="13"/>
+      <c r="J121" s="13"/>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" s="5"/>
@@ -2144,8 +2140,8 @@
       <c r="F122" s="5"/>
       <c r="G122" s="5"/>
       <c r="H122" s="5"/>
-      <c r="I122" s="15"/>
-      <c r="J122" s="15"/>
+      <c r="I122" s="13"/>
+      <c r="J122" s="13"/>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A123" s="5"/>
@@ -2156,8 +2152,8 @@
       <c r="F123" s="5"/>
       <c r="G123" s="5"/>
       <c r="H123" s="5"/>
-      <c r="I123" s="15"/>
-      <c r="J123" s="15"/>
+      <c r="I123" s="13"/>
+      <c r="J123" s="13"/>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A124" s="5"/>
@@ -2168,8 +2164,8 @@
       <c r="F124" s="5"/>
       <c r="G124" s="5"/>
       <c r="H124" s="5"/>
-      <c r="I124" s="15"/>
-      <c r="J124" s="15"/>
+      <c r="I124" s="13"/>
+      <c r="J124" s="13"/>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" s="5"/>
@@ -2180,8 +2176,8 @@
       <c r="F125" s="5"/>
       <c r="G125" s="5"/>
       <c r="H125" s="5"/>
-      <c r="I125" s="15"/>
-      <c r="J125" s="15"/>
+      <c r="I125" s="13"/>
+      <c r="J125" s="13"/>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" s="5"/>
@@ -2192,8 +2188,8 @@
       <c r="F126" s="5"/>
       <c r="G126" s="5"/>
       <c r="H126" s="5"/>
-      <c r="I126" s="15"/>
-      <c r="J126" s="15"/>
+      <c r="I126" s="13"/>
+      <c r="J126" s="13"/>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A127" s="5"/>
@@ -2204,8 +2200,8 @@
       <c r="F127" s="5"/>
       <c r="G127" s="5"/>
       <c r="H127" s="5"/>
-      <c r="I127" s="15"/>
-      <c r="J127" s="15"/>
+      <c r="I127" s="13"/>
+      <c r="J127" s="13"/>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A128" s="5"/>
@@ -2216,8 +2212,8 @@
       <c r="F128" s="5"/>
       <c r="G128" s="5"/>
       <c r="H128" s="5"/>
-      <c r="I128" s="15"/>
-      <c r="J128" s="15"/>
+      <c r="I128" s="13"/>
+      <c r="J128" s="13"/>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A129" s="5"/>
@@ -2228,8 +2224,8 @@
       <c r="F129" s="5"/>
       <c r="G129" s="5"/>
       <c r="H129" s="5"/>
-      <c r="I129" s="15"/>
-      <c r="J129" s="15"/>
+      <c r="I129" s="13"/>
+      <c r="J129" s="13"/>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A130" s="5"/>
@@ -2237,11 +2233,8 @@
       <c r="C130" s="5"/>
       <c r="D130" s="5"/>
       <c r="E130" s="5"/>
-      <c r="F130" s="14"/>
-      <c r="G130" s="14"/>
-      <c r="H130" s="12"/>
-      <c r="I130" s="13"/>
-      <c r="J130" s="13"/>
+      <c r="F130" s="12"/>
+      <c r="G130" s="12"/>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" s="5"/>
@@ -2251,9 +2244,6 @@
       <c r="E131" s="5"/>
       <c r="F131" s="5"/>
       <c r="G131" s="5"/>
-      <c r="H131" s="12"/>
-      <c r="I131" s="13"/>
-      <c r="J131" s="13"/>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A132" s="5"/>
@@ -2263,9 +2253,6 @@
       <c r="E132" s="5"/>
       <c r="F132" s="5"/>
       <c r="G132" s="5"/>
-      <c r="H132" s="12"/>
-      <c r="I132" s="13"/>
-      <c r="J132" s="13"/>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A133" s="5"/>
@@ -2275,9 +2262,6 @@
       <c r="E133" s="5"/>
       <c r="F133" s="5"/>
       <c r="G133" s="5"/>
-      <c r="H133" s="12"/>
-      <c r="I133" s="13"/>
-      <c r="J133" s="13"/>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A134" s="5"/>
@@ -2287,9 +2271,6 @@
       <c r="E134" s="5"/>
       <c r="F134" s="5"/>
       <c r="G134" s="5"/>
-      <c r="H134" s="12"/>
-      <c r="I134" s="13"/>
-      <c r="J134" s="13"/>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A135" s="5"/>
@@ -2299,9 +2280,6 @@
       <c r="E135" s="5"/>
       <c r="F135" s="5"/>
       <c r="G135" s="5"/>
-      <c r="H135" s="12"/>
-      <c r="I135" s="13"/>
-      <c r="J135" s="13"/>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A136" s="5"/>
@@ -2311,9 +2289,6 @@
       <c r="E136" s="5"/>
       <c r="F136" s="5"/>
       <c r="G136" s="5"/>
-      <c r="H136" s="12"/>
-      <c r="I136" s="13"/>
-      <c r="J136" s="13"/>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A137" s="5"/>
@@ -2323,9 +2298,6 @@
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
       <c r="G137" s="5"/>
-      <c r="H137" s="12"/>
-      <c r="I137" s="13"/>
-      <c r="J137" s="13"/>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" s="5"/>
@@ -2335,9 +2307,6 @@
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
       <c r="G138" s="5"/>
-      <c r="H138" s="12"/>
-      <c r="I138" s="13"/>
-      <c r="J138" s="13"/>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" s="5"/>
@@ -2347,9 +2316,6 @@
       <c r="E139" s="5"/>
       <c r="F139" s="5"/>
       <c r="G139" s="5"/>
-      <c r="H139" s="12"/>
-      <c r="I139" s="13"/>
-      <c r="J139" s="13"/>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A140" s="5"/>
@@ -2359,9 +2325,6 @@
       <c r="E140" s="5"/>
       <c r="F140" s="5"/>
       <c r="G140" s="5"/>
-      <c r="H140" s="12"/>
-      <c r="I140" s="13"/>
-      <c r="J140" s="13"/>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A141" s="5"/>
@@ -2371,9 +2334,6 @@
       <c r="E141" s="5"/>
       <c r="F141" s="5"/>
       <c r="G141" s="5"/>
-      <c r="H141" s="12"/>
-      <c r="I141" s="13"/>
-      <c r="J141" s="13"/>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A142" s="5"/>
@@ -2383,9 +2343,6 @@
       <c r="E142" s="5"/>
       <c r="F142" s="5"/>
       <c r="G142" s="5"/>
-      <c r="H142" s="12"/>
-      <c r="I142" s="13"/>
-      <c r="J142" s="13"/>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A143" s="5"/>
@@ -2395,9 +2352,6 @@
       <c r="E143" s="5"/>
       <c r="F143" s="5"/>
       <c r="G143" s="5"/>
-      <c r="H143" s="12"/>
-      <c r="I143" s="13"/>
-      <c r="J143" s="13"/>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A144" s="5"/>
@@ -2407,11 +2361,8 @@
       <c r="E144" s="5"/>
       <c r="F144" s="5"/>
       <c r="G144" s="5"/>
-      <c r="H144" s="12"/>
-      <c r="I144" s="13"/>
-      <c r="J144" s="13"/>
-    </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A145" s="5"/>
       <c r="B145" s="5"/>
       <c r="C145" s="5"/>
@@ -2419,11 +2370,8 @@
       <c r="E145" s="5"/>
       <c r="F145" s="5"/>
       <c r="G145" s="5"/>
-      <c r="H145" s="12"/>
-      <c r="I145" s="13"/>
-      <c r="J145" s="13"/>
-    </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146" s="5"/>
       <c r="B146" s="5"/>
       <c r="C146" s="5"/>
@@ -2431,11 +2379,8 @@
       <c r="E146" s="5"/>
       <c r="F146" s="5"/>
       <c r="G146" s="5"/>
-      <c r="H146" s="12"/>
-      <c r="I146" s="13"/>
-      <c r="J146" s="13"/>
-    </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147" s="5"/>
       <c r="B147" s="5"/>
       <c r="C147" s="5"/>
@@ -2443,11 +2388,8 @@
       <c r="E147" s="5"/>
       <c r="F147" s="5"/>
       <c r="G147" s="5"/>
-      <c r="H147" s="12"/>
-      <c r="I147" s="13"/>
-      <c r="J147" s="13"/>
-    </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" s="5"/>
       <c r="B148" s="5"/>
       <c r="C148" s="5"/>
@@ -2455,11 +2397,8 @@
       <c r="E148" s="5"/>
       <c r="F148" s="5"/>
       <c r="G148" s="5"/>
-      <c r="H148" s="12"/>
-      <c r="I148" s="13"/>
-      <c r="J148" s="13"/>
-    </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149" s="5"/>
       <c r="B149" s="5"/>
       <c r="C149" s="5"/>
@@ -2467,11 +2406,8 @@
       <c r="E149" s="5"/>
       <c r="F149" s="5"/>
       <c r="G149" s="5"/>
-      <c r="H149" s="12"/>
-      <c r="I149" s="13"/>
-      <c r="J149" s="13"/>
-    </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" s="5"/>
       <c r="B150" s="5"/>
       <c r="C150" s="5"/>
@@ -2479,11 +2415,8 @@
       <c r="E150" s="5"/>
       <c r="F150" s="5"/>
       <c r="G150" s="5"/>
-      <c r="H150" s="12"/>
-      <c r="I150" s="13"/>
-      <c r="J150" s="13"/>
-    </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151" s="5"/>
       <c r="B151" s="5"/>
       <c r="C151" s="5"/>
@@ -2491,11 +2424,8 @@
       <c r="E151" s="5"/>
       <c r="F151" s="5"/>
       <c r="G151" s="5"/>
-      <c r="H151" s="12"/>
-      <c r="I151" s="13"/>
-      <c r="J151" s="13"/>
-    </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" s="5"/>
       <c r="B152" s="5"/>
       <c r="C152" s="5"/>
@@ -2503,11 +2433,8 @@
       <c r="E152" s="5"/>
       <c r="F152" s="5"/>
       <c r="G152" s="5"/>
-      <c r="H152" s="12"/>
-      <c r="I152" s="13"/>
-      <c r="J152" s="13"/>
-    </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A153" s="5"/>
       <c r="B153" s="5"/>
       <c r="C153" s="5"/>
@@ -2515,11 +2442,8 @@
       <c r="E153" s="5"/>
       <c r="F153" s="5"/>
       <c r="G153" s="5"/>
-      <c r="H153" s="12"/>
-      <c r="I153" s="13"/>
-      <c r="J153" s="13"/>
-    </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A154" s="5"/>
       <c r="B154" s="5"/>
       <c r="C154" s="5"/>
@@ -2527,11 +2451,8 @@
       <c r="E154" s="5"/>
       <c r="F154" s="5"/>
       <c r="G154" s="5"/>
-      <c r="H154" s="12"/>
-      <c r="I154" s="13"/>
-      <c r="J154" s="13"/>
-    </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A155" s="5"/>
       <c r="B155" s="5"/>
       <c r="C155" s="5"/>
@@ -2539,11 +2460,8 @@
       <c r="E155" s="5"/>
       <c r="F155" s="5"/>
       <c r="G155" s="5"/>
-      <c r="H155" s="12"/>
-      <c r="I155" s="13"/>
-      <c r="J155" s="13"/>
-    </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156" s="5"/>
       <c r="B156" s="5"/>
       <c r="C156" s="5"/>
@@ -2551,11 +2469,8 @@
       <c r="E156" s="5"/>
       <c r="F156" s="5"/>
       <c r="G156" s="5"/>
-      <c r="H156" s="12"/>
-      <c r="I156" s="13"/>
-      <c r="J156" s="13"/>
-    </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A157" s="5"/>
       <c r="B157" s="5"/>
       <c r="C157" s="5"/>
@@ -2563,11 +2478,8 @@
       <c r="E157" s="5"/>
       <c r="F157" s="5"/>
       <c r="G157" s="5"/>
-      <c r="H157" s="12"/>
-      <c r="I157" s="13"/>
-      <c r="J157" s="13"/>
-    </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" s="5"/>
       <c r="B158" s="5"/>
       <c r="C158" s="5"/>
@@ -2575,11 +2487,8 @@
       <c r="E158" s="5"/>
       <c r="F158" s="5"/>
       <c r="G158" s="5"/>
-      <c r="H158" s="12"/>
-      <c r="I158" s="13"/>
-      <c r="J158" s="13"/>
-    </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A159" s="5"/>
       <c r="B159" s="5"/>
       <c r="C159" s="5"/>
@@ -2587,11 +2496,8 @@
       <c r="E159" s="5"/>
       <c r="F159" s="5"/>
       <c r="G159" s="5"/>
-      <c r="H159" s="12"/>
-      <c r="I159" s="13"/>
-      <c r="J159" s="13"/>
-    </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A160" s="5"/>
       <c r="B160" s="5"/>
       <c r="C160" s="5"/>
@@ -2599,11 +2505,8 @@
       <c r="E160" s="5"/>
       <c r="F160" s="5"/>
       <c r="G160" s="5"/>
-      <c r="H160" s="12"/>
-      <c r="I160" s="13"/>
-      <c r="J160" s="13"/>
-    </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A161" s="5"/>
       <c r="B161" s="5"/>
       <c r="C161" s="5"/>
@@ -2611,11 +2514,8 @@
       <c r="E161" s="5"/>
       <c r="F161" s="5"/>
       <c r="G161" s="5"/>
-      <c r="H161" s="12"/>
-      <c r="I161" s="13"/>
-      <c r="J161" s="13"/>
-    </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A162" s="5"/>
       <c r="B162" s="5"/>
       <c r="C162" s="5"/>
@@ -2623,11 +2523,8 @@
       <c r="E162" s="5"/>
       <c r="F162" s="5"/>
       <c r="G162" s="5"/>
-      <c r="H162" s="12"/>
-      <c r="I162" s="13"/>
-      <c r="J162" s="13"/>
-    </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A163" s="5"/>
       <c r="B163" s="5"/>
       <c r="C163" s="5"/>
@@ -2635,11 +2532,8 @@
       <c r="E163" s="5"/>
       <c r="F163" s="5"/>
       <c r="G163" s="5"/>
-      <c r="H163" s="12"/>
-      <c r="I163" s="13"/>
-      <c r="J163" s="13"/>
-    </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A164" s="5"/>
       <c r="B164" s="5"/>
       <c r="C164" s="5"/>
@@ -2647,11 +2541,8 @@
       <c r="E164" s="5"/>
       <c r="F164" s="5"/>
       <c r="G164" s="5"/>
-      <c r="H164" s="12"/>
-      <c r="I164" s="13"/>
-      <c r="J164" s="13"/>
-    </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A165" s="5"/>
       <c r="B165" s="5"/>
       <c r="C165" s="5"/>
@@ -2659,11 +2550,8 @@
       <c r="E165" s="5"/>
       <c r="F165" s="5"/>
       <c r="G165" s="5"/>
-      <c r="H165" s="12"/>
-      <c r="I165" s="13"/>
-      <c r="J165" s="13"/>
-    </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A166" s="5"/>
       <c r="B166" s="5"/>
       <c r="C166" s="5"/>
@@ -2671,11 +2559,8 @@
       <c r="E166" s="5"/>
       <c r="F166" s="5"/>
       <c r="G166" s="5"/>
-      <c r="H166" s="12"/>
-      <c r="I166" s="13"/>
-      <c r="J166" s="13"/>
-    </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A167" s="5"/>
       <c r="B167" s="5"/>
       <c r="C167" s="5"/>
@@ -2683,11 +2568,8 @@
       <c r="E167" s="5"/>
       <c r="F167" s="5"/>
       <c r="G167" s="5"/>
-      <c r="H167" s="12"/>
-      <c r="I167" s="13"/>
-      <c r="J167" s="13"/>
-    </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A168" s="5"/>
       <c r="B168" s="5"/>
       <c r="C168" s="5"/>
@@ -2695,11 +2577,8 @@
       <c r="E168" s="5"/>
       <c r="F168" s="5"/>
       <c r="G168" s="5"/>
-      <c r="H168" s="12"/>
-      <c r="I168" s="13"/>
-      <c r="J168" s="13"/>
-    </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A169" s="5"/>
       <c r="B169" s="5"/>
       <c r="C169" s="5"/>
@@ -2707,11 +2586,8 @@
       <c r="E169" s="5"/>
       <c r="F169" s="5"/>
       <c r="G169" s="5"/>
-      <c r="H169" s="12"/>
-      <c r="I169" s="13"/>
-      <c r="J169" s="13"/>
-    </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A170" s="5"/>
       <c r="B170" s="5"/>
       <c r="C170" s="5"/>
@@ -2719,11 +2595,8 @@
       <c r="E170" s="5"/>
       <c r="F170" s="5"/>
       <c r="G170" s="5"/>
-      <c r="H170" s="12"/>
-      <c r="I170" s="13"/>
-      <c r="J170" s="13"/>
-    </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A171" s="5"/>
       <c r="B171" s="5"/>
       <c r="C171" s="5"/>
@@ -2731,11 +2604,8 @@
       <c r="E171" s="5"/>
       <c r="F171" s="5"/>
       <c r="G171" s="5"/>
-      <c r="H171" s="12"/>
-      <c r="I171" s="13"/>
-      <c r="J171" s="13"/>
-    </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A172" s="5"/>
       <c r="B172" s="5"/>
       <c r="C172" s="5"/>
@@ -2743,11 +2613,8 @@
       <c r="E172" s="5"/>
       <c r="F172" s="5"/>
       <c r="G172" s="5"/>
-      <c r="H172" s="12"/>
-      <c r="I172" s="13"/>
-      <c r="J172" s="13"/>
-    </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A173" s="5"/>
       <c r="B173" s="5"/>
       <c r="C173" s="5"/>
@@ -2755,11 +2622,8 @@
       <c r="E173" s="5"/>
       <c r="F173" s="5"/>
       <c r="G173" s="5"/>
-      <c r="H173" s="12"/>
-      <c r="I173" s="13"/>
-      <c r="J173" s="13"/>
-    </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A174" s="5"/>
       <c r="B174" s="5"/>
       <c r="C174" s="5"/>
@@ -2767,11 +2631,8 @@
       <c r="E174" s="5"/>
       <c r="F174" s="5"/>
       <c r="G174" s="5"/>
-      <c r="H174" s="12"/>
-      <c r="I174" s="13"/>
-      <c r="J174" s="13"/>
-    </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A175" s="5"/>
       <c r="B175" s="5"/>
       <c r="C175" s="5"/>
@@ -2779,11 +2640,8 @@
       <c r="E175" s="5"/>
       <c r="F175" s="5"/>
       <c r="G175" s="5"/>
-      <c r="H175" s="12"/>
-      <c r="I175" s="13"/>
-      <c r="J175" s="13"/>
-    </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A176" s="5"/>
       <c r="B176" s="5"/>
       <c r="C176" s="5"/>
@@ -2791,11 +2649,8 @@
       <c r="E176" s="5"/>
       <c r="F176" s="5"/>
       <c r="G176" s="5"/>
-      <c r="H176" s="12"/>
-      <c r="I176" s="13"/>
-      <c r="J176" s="13"/>
-    </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A177" s="5"/>
       <c r="B177" s="5"/>
       <c r="C177" s="5"/>
@@ -2803,11 +2658,8 @@
       <c r="E177" s="5"/>
       <c r="F177" s="5"/>
       <c r="G177" s="5"/>
-      <c r="H177" s="12"/>
-      <c r="I177" s="13"/>
-      <c r="J177" s="13"/>
-    </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A178" s="5"/>
       <c r="B178" s="5"/>
       <c r="C178" s="5"/>
@@ -2815,11 +2667,8 @@
       <c r="E178" s="5"/>
       <c r="F178" s="5"/>
       <c r="G178" s="5"/>
-      <c r="H178" s="12"/>
-      <c r="I178" s="13"/>
-      <c r="J178" s="13"/>
-    </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A179" s="5"/>
       <c r="B179" s="5"/>
       <c r="C179" s="5"/>
@@ -2827,11 +2676,8 @@
       <c r="E179" s="5"/>
       <c r="F179" s="5"/>
       <c r="G179" s="5"/>
-      <c r="H179" s="12"/>
-      <c r="I179" s="13"/>
-      <c r="J179" s="13"/>
-    </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A180" s="5"/>
       <c r="B180" s="5"/>
       <c r="C180" s="5"/>
@@ -2839,11 +2685,8 @@
       <c r="E180" s="5"/>
       <c r="F180" s="5"/>
       <c r="G180" s="5"/>
-      <c r="H180" s="12"/>
-      <c r="I180" s="13"/>
-      <c r="J180" s="13"/>
-    </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A181" s="5"/>
       <c r="B181" s="5"/>
       <c r="C181" s="5"/>
@@ -2851,11 +2694,8 @@
       <c r="E181" s="5"/>
       <c r="F181" s="5"/>
       <c r="G181" s="5"/>
-      <c r="H181" s="12"/>
-      <c r="I181" s="13"/>
-      <c r="J181" s="13"/>
-    </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A182" s="5"/>
       <c r="B182" s="5"/>
       <c r="C182" s="5"/>
@@ -2863,11 +2703,8 @@
       <c r="E182" s="5"/>
       <c r="F182" s="5"/>
       <c r="G182" s="5"/>
-      <c r="H182" s="12"/>
-      <c r="I182" s="13"/>
-      <c r="J182" s="13"/>
-    </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A183" s="5"/>
       <c r="B183" s="5"/>
       <c r="C183" s="5"/>
@@ -2875,11 +2712,8 @@
       <c r="E183" s="5"/>
       <c r="F183" s="5"/>
       <c r="G183" s="5"/>
-      <c r="H183" s="12"/>
-      <c r="I183" s="13"/>
-      <c r="J183" s="13"/>
-    </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A184" s="5"/>
       <c r="B184" s="5"/>
       <c r="C184" s="5"/>
@@ -2887,11 +2721,8 @@
       <c r="E184" s="5"/>
       <c r="F184" s="5"/>
       <c r="G184" s="5"/>
-      <c r="H184" s="12"/>
-      <c r="I184" s="13"/>
-      <c r="J184" s="13"/>
-    </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A185" s="5"/>
       <c r="B185" s="5"/>
       <c r="C185" s="5"/>
@@ -2899,11 +2730,8 @@
       <c r="E185" s="5"/>
       <c r="F185" s="5"/>
       <c r="G185" s="5"/>
-      <c r="H185" s="12"/>
-      <c r="I185" s="13"/>
-      <c r="J185" s="13"/>
-    </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A186" s="5"/>
       <c r="B186" s="5"/>
       <c r="C186" s="5"/>
@@ -2911,11 +2739,8 @@
       <c r="E186" s="5"/>
       <c r="F186" s="5"/>
       <c r="G186" s="5"/>
-      <c r="H186" s="12"/>
-      <c r="I186" s="13"/>
-      <c r="J186" s="13"/>
-    </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A187" s="5"/>
       <c r="B187" s="5"/>
       <c r="C187" s="5"/>
@@ -2923,11 +2748,8 @@
       <c r="E187" s="5"/>
       <c r="F187" s="5"/>
       <c r="G187" s="5"/>
-      <c r="H187" s="12"/>
-      <c r="I187" s="13"/>
-      <c r="J187" s="13"/>
-    </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A188" s="5"/>
       <c r="B188" s="5"/>
       <c r="C188" s="5"/>
@@ -2935,11 +2757,8 @@
       <c r="E188" s="5"/>
       <c r="F188" s="5"/>
       <c r="G188" s="5"/>
-      <c r="H188" s="12"/>
-      <c r="I188" s="13"/>
-      <c r="J188" s="13"/>
-    </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A189" s="5"/>
       <c r="B189" s="5"/>
       <c r="C189" s="5"/>
@@ -2947,11 +2766,8 @@
       <c r="E189" s="5"/>
       <c r="F189" s="5"/>
       <c r="G189" s="5"/>
-      <c r="H189" s="12"/>
-      <c r="I189" s="13"/>
-      <c r="J189" s="13"/>
-    </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A190" s="5"/>
       <c r="B190" s="5"/>
       <c r="C190" s="5"/>
@@ -2959,11 +2775,8 @@
       <c r="E190" s="5"/>
       <c r="F190" s="5"/>
       <c r="G190" s="5"/>
-      <c r="H190" s="12"/>
-      <c r="I190" s="13"/>
-      <c r="J190" s="13"/>
-    </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A191" s="5"/>
       <c r="B191" s="5"/>
       <c r="C191" s="5"/>
@@ -2971,11 +2784,8 @@
       <c r="E191" s="5"/>
       <c r="F191" s="5"/>
       <c r="G191" s="5"/>
-      <c r="H191" s="12"/>
-      <c r="I191" s="13"/>
-      <c r="J191" s="13"/>
-    </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A192" s="5"/>
       <c r="B192" s="5"/>
       <c r="C192" s="5"/>
@@ -2983,11 +2793,8 @@
       <c r="E192" s="5"/>
       <c r="F192" s="5"/>
       <c r="G192" s="5"/>
-      <c r="H192" s="12"/>
-      <c r="I192" s="13"/>
-      <c r="J192" s="13"/>
-    </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A193" s="5"/>
       <c r="B193" s="5"/>
       <c r="C193" s="5"/>
@@ -2995,11 +2802,8 @@
       <c r="E193" s="5"/>
       <c r="F193" s="5"/>
       <c r="G193" s="5"/>
-      <c r="H193" s="12"/>
-      <c r="I193" s="13"/>
-      <c r="J193" s="13"/>
-    </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A194" s="5"/>
       <c r="B194" s="5"/>
       <c r="C194" s="5"/>
@@ -3007,11 +2811,8 @@
       <c r="E194" s="5"/>
       <c r="F194" s="5"/>
       <c r="G194" s="5"/>
-      <c r="H194" s="12"/>
-      <c r="I194" s="13"/>
-      <c r="J194" s="13"/>
-    </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A195" s="5"/>
       <c r="B195" s="5"/>
       <c r="C195" s="5"/>
@@ -3019,11 +2820,8 @@
       <c r="E195" s="5"/>
       <c r="F195" s="5"/>
       <c r="G195" s="5"/>
-      <c r="H195" s="12"/>
-      <c r="I195" s="13"/>
-      <c r="J195" s="13"/>
-    </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A196" s="5"/>
       <c r="B196" s="5"/>
       <c r="C196" s="5"/>
@@ -3031,11 +2829,8 @@
       <c r="E196" s="5"/>
       <c r="F196" s="5"/>
       <c r="G196" s="5"/>
-      <c r="H196" s="12"/>
-      <c r="I196" s="13"/>
-      <c r="J196" s="13"/>
-    </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A197" s="5"/>
       <c r="B197" s="5"/>
       <c r="C197" s="5"/>
@@ -3043,11 +2838,8 @@
       <c r="E197" s="5"/>
       <c r="F197" s="5"/>
       <c r="G197" s="5"/>
-      <c r="H197" s="12"/>
-      <c r="I197" s="13"/>
-      <c r="J197" s="13"/>
-    </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="198" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A198" s="5"/>
       <c r="B198" s="5"/>
       <c r="C198" s="5"/>
@@ -3055,11 +2847,8 @@
       <c r="E198" s="5"/>
       <c r="F198" s="5"/>
       <c r="G198" s="5"/>
-      <c r="H198" s="12"/>
-      <c r="I198" s="13"/>
-      <c r="J198" s="13"/>
-    </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A199" s="5"/>
       <c r="B199" s="5"/>
       <c r="C199" s="5"/>
@@ -3067,11 +2856,8 @@
       <c r="E199" s="5"/>
       <c r="F199" s="5"/>
       <c r="G199" s="5"/>
-      <c r="H199" s="12"/>
-      <c r="I199" s="13"/>
-      <c r="J199" s="13"/>
-    </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A200" s="5"/>
       <c r="B200" s="5"/>
       <c r="C200" s="5"/>
@@ -3079,11 +2865,8 @@
       <c r="E200" s="5"/>
       <c r="F200" s="5"/>
       <c r="G200" s="5"/>
-      <c r="H200" s="12"/>
-      <c r="I200" s="13"/>
-      <c r="J200" s="13"/>
-    </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A201" s="5"/>
       <c r="B201" s="5"/>
       <c r="C201" s="5"/>
@@ -3091,11 +2874,8 @@
       <c r="E201" s="5"/>
       <c r="F201" s="5"/>
       <c r="G201" s="5"/>
-      <c r="H201" s="12"/>
-      <c r="I201" s="13"/>
-      <c r="J201" s="13"/>
-    </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A202" s="5"/>
       <c r="B202" s="5"/>
       <c r="C202" s="5"/>
@@ -3103,11 +2883,8 @@
       <c r="E202" s="5"/>
       <c r="F202" s="5"/>
       <c r="G202" s="5"/>
-      <c r="H202" s="12"/>
-      <c r="I202" s="13"/>
-      <c r="J202" s="13"/>
-    </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A203" s="5"/>
       <c r="B203" s="5"/>
       <c r="C203" s="5"/>
@@ -3115,11 +2892,8 @@
       <c r="E203" s="5"/>
       <c r="F203" s="5"/>
       <c r="G203" s="5"/>
-      <c r="H203" s="12"/>
-      <c r="I203" s="13"/>
-      <c r="J203" s="13"/>
-    </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A204" s="5"/>
       <c r="B204" s="5"/>
       <c r="C204" s="5"/>
@@ -3127,11 +2901,8 @@
       <c r="E204" s="5"/>
       <c r="F204" s="5"/>
       <c r="G204" s="5"/>
-      <c r="H204" s="12"/>
-      <c r="I204" s="13"/>
-      <c r="J204" s="13"/>
-    </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A205" s="5"/>
       <c r="B205" s="5"/>
       <c r="C205" s="5"/>
@@ -3139,11 +2910,8 @@
       <c r="E205" s="5"/>
       <c r="F205" s="5"/>
       <c r="G205" s="5"/>
-      <c r="H205" s="12"/>
-      <c r="I205" s="13"/>
-      <c r="J205" s="13"/>
-    </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A206" s="5"/>
       <c r="B206" s="5"/>
       <c r="C206" s="5"/>
@@ -3151,11 +2919,8 @@
       <c r="E206" s="5"/>
       <c r="F206" s="5"/>
       <c r="G206" s="5"/>
-      <c r="H206" s="12"/>
-      <c r="I206" s="13"/>
-      <c r="J206" s="13"/>
-    </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A207" s="5"/>
       <c r="B207" s="5"/>
       <c r="C207" s="5"/>
@@ -3163,11 +2928,8 @@
       <c r="E207" s="5"/>
       <c r="F207" s="5"/>
       <c r="G207" s="5"/>
-      <c r="H207" s="12"/>
-      <c r="I207" s="13"/>
-      <c r="J207" s="13"/>
-    </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A208" s="5"/>
       <c r="B208" s="5"/>
       <c r="C208" s="5"/>
@@ -3175,11 +2937,8 @@
       <c r="E208" s="5"/>
       <c r="F208" s="5"/>
       <c r="G208" s="5"/>
-      <c r="H208" s="12"/>
-      <c r="I208" s="13"/>
-      <c r="J208" s="13"/>
-    </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A209" s="5"/>
       <c r="B209" s="5"/>
       <c r="C209" s="5"/>
@@ -3187,11 +2946,8 @@
       <c r="E209" s="5"/>
       <c r="F209" s="5"/>
       <c r="G209" s="5"/>
-      <c r="H209" s="12"/>
-      <c r="I209" s="13"/>
-      <c r="J209" s="13"/>
-    </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="210" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A210" s="5"/>
       <c r="B210" s="5"/>
       <c r="C210" s="5"/>
@@ -3199,11 +2955,8 @@
       <c r="E210" s="5"/>
       <c r="F210" s="5"/>
       <c r="G210" s="5"/>
-      <c r="H210" s="12"/>
-      <c r="I210" s="13"/>
-      <c r="J210" s="13"/>
-    </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A211" s="5"/>
       <c r="B211" s="5"/>
       <c r="C211" s="5"/>
@@ -3211,11 +2964,8 @@
       <c r="E211" s="5"/>
       <c r="F211" s="5"/>
       <c r="G211" s="5"/>
-      <c r="H211" s="12"/>
-      <c r="I211" s="13"/>
-      <c r="J211" s="13"/>
-    </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A212" s="5"/>
       <c r="B212" s="5"/>
       <c r="C212" s="5"/>
@@ -3223,11 +2973,8 @@
       <c r="E212" s="5"/>
       <c r="F212" s="5"/>
       <c r="G212" s="5"/>
-      <c r="H212" s="12"/>
-      <c r="I212" s="13"/>
-      <c r="J212" s="13"/>
-    </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="213" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A213" s="5"/>
       <c r="B213" s="5"/>
       <c r="C213" s="5"/>
@@ -3235,11 +2982,8 @@
       <c r="E213" s="5"/>
       <c r="F213" s="5"/>
       <c r="G213" s="5"/>
-      <c r="H213" s="12"/>
-      <c r="I213" s="13"/>
-      <c r="J213" s="13"/>
-    </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="214" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A214" s="5"/>
       <c r="B214" s="5"/>
       <c r="C214" s="5"/>
@@ -3247,11 +2991,8 @@
       <c r="E214" s="5"/>
       <c r="F214" s="5"/>
       <c r="G214" s="5"/>
-      <c r="H214" s="12"/>
-      <c r="I214" s="13"/>
-      <c r="J214" s="13"/>
-    </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="215" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A215" s="5"/>
       <c r="B215" s="5"/>
       <c r="C215" s="5"/>
@@ -3259,11 +3000,8 @@
       <c r="E215" s="5"/>
       <c r="F215" s="5"/>
       <c r="G215" s="5"/>
-      <c r="H215" s="12"/>
-      <c r="I215" s="13"/>
-      <c r="J215" s="13"/>
-    </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="216" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A216" s="5"/>
       <c r="B216" s="5"/>
       <c r="C216" s="5"/>
@@ -3271,11 +3009,8 @@
       <c r="E216" s="5"/>
       <c r="F216" s="5"/>
       <c r="G216" s="5"/>
-      <c r="H216" s="12"/>
-      <c r="I216" s="13"/>
-      <c r="J216" s="13"/>
-    </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A217" s="5"/>
       <c r="B217" s="5"/>
       <c r="C217" s="5"/>
@@ -3283,11 +3018,8 @@
       <c r="E217" s="5"/>
       <c r="F217" s="5"/>
       <c r="G217" s="5"/>
-      <c r="H217" s="12"/>
-      <c r="I217" s="13"/>
-      <c r="J217" s="13"/>
-    </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A218" s="5"/>
       <c r="B218" s="5"/>
       <c r="C218" s="5"/>
@@ -3295,11 +3027,8 @@
       <c r="E218" s="5"/>
       <c r="F218" s="5"/>
       <c r="G218" s="5"/>
-      <c r="H218" s="12"/>
-      <c r="I218" s="13"/>
-      <c r="J218" s="13"/>
-    </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="219" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A219" s="5"/>
       <c r="B219" s="5"/>
       <c r="C219" s="5"/>
@@ -3307,11 +3036,8 @@
       <c r="E219" s="5"/>
       <c r="F219" s="5"/>
       <c r="G219" s="5"/>
-      <c r="H219" s="12"/>
-      <c r="I219" s="13"/>
-      <c r="J219" s="13"/>
-    </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A220" s="5"/>
       <c r="B220" s="5"/>
       <c r="C220" s="5"/>
@@ -3319,11 +3045,8 @@
       <c r="E220" s="5"/>
       <c r="F220" s="5"/>
       <c r="G220" s="5"/>
-      <c r="H220" s="12"/>
-      <c r="I220" s="13"/>
-      <c r="J220" s="13"/>
-    </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="221" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A221" s="5"/>
       <c r="B221" s="5"/>
       <c r="C221" s="5"/>
@@ -3331,11 +3054,8 @@
       <c r="E221" s="5"/>
       <c r="F221" s="5"/>
       <c r="G221" s="5"/>
-      <c r="H221" s="12"/>
-      <c r="I221" s="13"/>
-      <c r="J221" s="13"/>
-    </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A222" s="5"/>
       <c r="B222" s="5"/>
       <c r="C222" s="5"/>
@@ -3343,11 +3063,8 @@
       <c r="E222" s="5"/>
       <c r="F222" s="5"/>
       <c r="G222" s="5"/>
-      <c r="H222" s="12"/>
-      <c r="I222" s="13"/>
-      <c r="J222" s="13"/>
-    </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A223" s="5"/>
       <c r="B223" s="5"/>
       <c r="C223" s="5"/>
@@ -3355,11 +3072,8 @@
       <c r="E223" s="5"/>
       <c r="F223" s="5"/>
       <c r="G223" s="5"/>
-      <c r="H223" s="12"/>
-      <c r="I223" s="13"/>
-      <c r="J223" s="13"/>
-    </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A224" s="5"/>
       <c r="B224" s="5"/>
       <c r="C224" s="5"/>
@@ -3367,11 +3081,8 @@
       <c r="E224" s="5"/>
       <c r="F224" s="5"/>
       <c r="G224" s="5"/>
-      <c r="H224" s="12"/>
-      <c r="I224" s="13"/>
-      <c r="J224" s="13"/>
-    </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A225" s="5"/>
       <c r="B225" s="5"/>
       <c r="C225" s="5"/>
@@ -3379,11 +3090,8 @@
       <c r="E225" s="5"/>
       <c r="F225" s="5"/>
       <c r="G225" s="5"/>
-      <c r="H225" s="12"/>
-      <c r="I225" s="13"/>
-      <c r="J225" s="13"/>
-    </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A226" s="5"/>
       <c r="B226" s="5"/>
       <c r="C226" s="5"/>
@@ -3391,11 +3099,8 @@
       <c r="E226" s="5"/>
       <c r="F226" s="5"/>
       <c r="G226" s="5"/>
-      <c r="H226" s="12"/>
-      <c r="I226" s="13"/>
-      <c r="J226" s="13"/>
-    </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A227" s="5"/>
       <c r="B227" s="5"/>
       <c r="C227" s="5"/>
@@ -3403,11 +3108,8 @@
       <c r="E227" s="5"/>
       <c r="F227" s="5"/>
       <c r="G227" s="5"/>
-      <c r="H227" s="12"/>
-      <c r="I227" s="13"/>
-      <c r="J227" s="13"/>
-    </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A228" s="5"/>
       <c r="B228" s="5"/>
       <c r="C228" s="5"/>
@@ -3415,11 +3117,8 @@
       <c r="E228" s="5"/>
       <c r="F228" s="5"/>
       <c r="G228" s="5"/>
-      <c r="H228" s="12"/>
-      <c r="I228" s="13"/>
-      <c r="J228" s="13"/>
-    </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A229" s="5"/>
       <c r="B229" s="5"/>
       <c r="C229" s="5"/>
@@ -3427,11 +3126,8 @@
       <c r="E229" s="5"/>
       <c r="F229" s="5"/>
       <c r="G229" s="5"/>
-      <c r="H229" s="12"/>
-      <c r="I229" s="13"/>
-      <c r="J229" s="13"/>
-    </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A230" s="5"/>
       <c r="B230" s="5"/>
       <c r="C230" s="5"/>
@@ -3439,11 +3135,8 @@
       <c r="E230" s="5"/>
       <c r="F230" s="5"/>
       <c r="G230" s="5"/>
-      <c r="H230" s="12"/>
-      <c r="I230" s="13"/>
-      <c r="J230" s="13"/>
-    </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A231" s="5"/>
       <c r="B231" s="5"/>
       <c r="C231" s="5"/>
@@ -3451,11 +3144,8 @@
       <c r="E231" s="5"/>
       <c r="F231" s="5"/>
       <c r="G231" s="5"/>
-      <c r="H231" s="12"/>
-      <c r="I231" s="13"/>
-      <c r="J231" s="13"/>
-    </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A232" s="5"/>
       <c r="B232" s="5"/>
       <c r="C232" s="5"/>
@@ -3463,11 +3153,8 @@
       <c r="E232" s="5"/>
       <c r="F232" s="5"/>
       <c r="G232" s="5"/>
-      <c r="H232" s="12"/>
-      <c r="I232" s="13"/>
-      <c r="J232" s="13"/>
-    </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A233" s="5"/>
       <c r="B233" s="5"/>
       <c r="C233" s="5"/>
@@ -3475,11 +3162,8 @@
       <c r="E233" s="5"/>
       <c r="F233" s="5"/>
       <c r="G233" s="5"/>
-      <c r="H233" s="12"/>
-      <c r="I233" s="13"/>
-      <c r="J233" s="13"/>
-    </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="234" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A234" s="5"/>
       <c r="B234" s="5"/>
       <c r="C234" s="5"/>
@@ -3487,11 +3171,8 @@
       <c r="E234" s="5"/>
       <c r="F234" s="5"/>
       <c r="G234" s="5"/>
-      <c r="H234" s="12"/>
-      <c r="I234" s="13"/>
-      <c r="J234" s="13"/>
-    </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A235" s="5"/>
       <c r="B235" s="5"/>
       <c r="C235" s="5"/>
@@ -3499,11 +3180,8 @@
       <c r="E235" s="5"/>
       <c r="F235" s="5"/>
       <c r="G235" s="5"/>
-      <c r="H235" s="12"/>
-      <c r="I235" s="13"/>
-      <c r="J235" s="13"/>
-    </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="236" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A236" s="5"/>
       <c r="B236" s="5"/>
       <c r="C236" s="5"/>
@@ -3511,11 +3189,8 @@
       <c r="E236" s="5"/>
       <c r="F236" s="5"/>
       <c r="G236" s="5"/>
-      <c r="H236" s="12"/>
-      <c r="I236" s="13"/>
-      <c r="J236" s="13"/>
-    </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A237" s="5"/>
       <c r="B237" s="5"/>
       <c r="C237" s="5"/>
@@ -3523,11 +3198,8 @@
       <c r="E237" s="5"/>
       <c r="F237" s="5"/>
       <c r="G237" s="5"/>
-      <c r="H237" s="12"/>
-      <c r="I237" s="13"/>
-      <c r="J237" s="13"/>
-    </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A238" s="5"/>
       <c r="B238" s="5"/>
       <c r="C238" s="5"/>
@@ -3535,11 +3207,8 @@
       <c r="E238" s="5"/>
       <c r="F238" s="5"/>
       <c r="G238" s="5"/>
-      <c r="H238" s="12"/>
-      <c r="I238" s="13"/>
-      <c r="J238" s="13"/>
-    </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="239" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A239" s="5"/>
       <c r="B239" s="5"/>
       <c r="C239" s="5"/>
@@ -3547,11 +3216,8 @@
       <c r="E239" s="5"/>
       <c r="F239" s="5"/>
       <c r="G239" s="5"/>
-      <c r="H239" s="12"/>
-      <c r="I239" s="13"/>
-      <c r="J239" s="13"/>
-    </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="240" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A240" s="5"/>
       <c r="B240" s="5"/>
       <c r="C240" s="5"/>
@@ -3559,11 +3225,8 @@
       <c r="E240" s="5"/>
       <c r="F240" s="5"/>
       <c r="G240" s="5"/>
-      <c r="H240" s="12"/>
-      <c r="I240" s="13"/>
-      <c r="J240" s="13"/>
-    </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="241" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A241" s="5"/>
       <c r="B241" s="5"/>
       <c r="C241" s="5"/>
@@ -3571,11 +3234,8 @@
       <c r="E241" s="5"/>
       <c r="F241" s="5"/>
       <c r="G241" s="5"/>
-      <c r="H241" s="12"/>
-      <c r="I241" s="13"/>
-      <c r="J241" s="13"/>
-    </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A242" s="5"/>
       <c r="B242" s="5"/>
       <c r="C242" s="5"/>
@@ -3583,11 +3243,8 @@
       <c r="E242" s="5"/>
       <c r="F242" s="5"/>
       <c r="G242" s="5"/>
-      <c r="H242" s="12"/>
-      <c r="I242" s="13"/>
-      <c r="J242" s="13"/>
-    </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="243" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A243" s="5"/>
       <c r="B243" s="5"/>
       <c r="C243" s="5"/>
@@ -3595,11 +3252,8 @@
       <c r="E243" s="5"/>
       <c r="F243" s="5"/>
       <c r="G243" s="5"/>
-      <c r="H243" s="12"/>
-      <c r="I243" s="13"/>
-      <c r="J243" s="13"/>
-    </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="244" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A244" s="5"/>
       <c r="B244" s="5"/>
       <c r="C244" s="5"/>
@@ -3607,11 +3261,8 @@
       <c r="E244" s="5"/>
       <c r="F244" s="5"/>
       <c r="G244" s="5"/>
-      <c r="H244" s="12"/>
-      <c r="I244" s="13"/>
-      <c r="J244" s="13"/>
-    </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="245" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A245" s="5"/>
       <c r="B245" s="5"/>
       <c r="C245" s="5"/>
@@ -3619,11 +3270,8 @@
       <c r="E245" s="5"/>
       <c r="F245" s="5"/>
       <c r="G245" s="5"/>
-      <c r="H245" s="12"/>
-      <c r="I245" s="13"/>
-      <c r="J245" s="13"/>
-    </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="246" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A246" s="5"/>
       <c r="B246" s="5"/>
       <c r="C246" s="5"/>
@@ -3631,11 +3279,8 @@
       <c r="E246" s="5"/>
       <c r="F246" s="5"/>
       <c r="G246" s="5"/>
-      <c r="H246" s="12"/>
-      <c r="I246" s="13"/>
-      <c r="J246" s="13"/>
-    </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="247" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A247" s="5"/>
       <c r="B247" s="5"/>
       <c r="C247" s="5"/>
@@ -3643,11 +3288,8 @@
       <c r="E247" s="5"/>
       <c r="F247" s="5"/>
       <c r="G247" s="5"/>
-      <c r="H247" s="12"/>
-      <c r="I247" s="13"/>
-      <c r="J247" s="13"/>
-    </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="248" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A248" s="5"/>
       <c r="B248" s="5"/>
       <c r="C248" s="5"/>
@@ -3655,11 +3297,8 @@
       <c r="E248" s="5"/>
       <c r="F248" s="5"/>
       <c r="G248" s="5"/>
-      <c r="H248" s="12"/>
-      <c r="I248" s="13"/>
-      <c r="J248" s="13"/>
-    </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="249" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A249" s="5"/>
       <c r="B249" s="5"/>
       <c r="C249" s="5"/>
@@ -3667,11 +3306,8 @@
       <c r="E249" s="5"/>
       <c r="F249" s="5"/>
       <c r="G249" s="5"/>
-      <c r="H249" s="12"/>
-      <c r="I249" s="13"/>
-      <c r="J249" s="13"/>
-    </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="250" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A250" s="5"/>
       <c r="B250" s="5"/>
       <c r="C250" s="5"/>
@@ -3679,11 +3315,8 @@
       <c r="E250" s="5"/>
       <c r="F250" s="5"/>
       <c r="G250" s="5"/>
-      <c r="H250" s="12"/>
-      <c r="I250" s="13"/>
-      <c r="J250" s="13"/>
-    </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="251" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A251" s="5"/>
       <c r="B251" s="5"/>
       <c r="C251" s="5"/>
@@ -3691,11 +3324,8 @@
       <c r="E251" s="5"/>
       <c r="F251" s="5"/>
       <c r="G251" s="5"/>
-      <c r="H251" s="12"/>
-      <c r="I251" s="13"/>
-      <c r="J251" s="13"/>
-    </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="252" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A252" s="5"/>
       <c r="B252" s="5"/>
       <c r="C252" s="5"/>
@@ -3703,11 +3333,8 @@
       <c r="E252" s="5"/>
       <c r="F252" s="5"/>
       <c r="G252" s="5"/>
-      <c r="H252" s="12"/>
-      <c r="I252" s="13"/>
-      <c r="J252" s="13"/>
-    </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="253" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A253" s="5"/>
       <c r="B253" s="5"/>
       <c r="C253" s="5"/>
@@ -3715,11 +3342,8 @@
       <c r="E253" s="5"/>
       <c r="F253" s="5"/>
       <c r="G253" s="5"/>
-      <c r="H253" s="12"/>
-      <c r="I253" s="13"/>
-      <c r="J253" s="13"/>
-    </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="254" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A254" s="5"/>
       <c r="B254" s="5"/>
       <c r="C254" s="5"/>
@@ -3727,11 +3351,8 @@
       <c r="E254" s="5"/>
       <c r="F254" s="5"/>
       <c r="G254" s="5"/>
-      <c r="H254" s="12"/>
-      <c r="I254" s="13"/>
-      <c r="J254" s="13"/>
-    </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="255" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A255" s="5"/>
       <c r="B255" s="5"/>
       <c r="C255" s="5"/>
@@ -3739,11 +3360,8 @@
       <c r="E255" s="5"/>
       <c r="F255" s="5"/>
       <c r="G255" s="5"/>
-      <c r="H255" s="12"/>
-      <c r="I255" s="13"/>
-      <c r="J255" s="13"/>
-    </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="256" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A256" s="5"/>
       <c r="B256" s="5"/>
       <c r="C256" s="5"/>
@@ -3751,11 +3369,8 @@
       <c r="E256" s="5"/>
       <c r="F256" s="5"/>
       <c r="G256" s="5"/>
-      <c r="H256" s="12"/>
-      <c r="I256" s="13"/>
-      <c r="J256" s="13"/>
-    </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="257" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A257" s="5"/>
       <c r="B257" s="5"/>
       <c r="C257" s="5"/>
@@ -3763,11 +3378,8 @@
       <c r="E257" s="5"/>
       <c r="F257" s="5"/>
       <c r="G257" s="5"/>
-      <c r="H257" s="12"/>
-      <c r="I257" s="13"/>
-      <c r="J257" s="13"/>
-    </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="258" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A258" s="5"/>
       <c r="B258" s="5"/>
       <c r="C258" s="5"/>
@@ -3775,11 +3387,8 @@
       <c r="E258" s="5"/>
       <c r="F258" s="5"/>
       <c r="G258" s="5"/>
-      <c r="H258" s="12"/>
-      <c r="I258" s="13"/>
-      <c r="J258" s="13"/>
-    </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A259" s="5"/>
       <c r="B259" s="5"/>
       <c r="C259" s="5"/>
@@ -3787,11 +3396,8 @@
       <c r="E259" s="5"/>
       <c r="F259" s="5"/>
       <c r="G259" s="5"/>
-      <c r="H259" s="12"/>
-      <c r="I259" s="13"/>
-      <c r="J259" s="13"/>
-    </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A260" s="5"/>
       <c r="B260" s="5"/>
       <c r="C260" s="5"/>
@@ -3799,11 +3405,8 @@
       <c r="E260" s="5"/>
       <c r="F260" s="5"/>
       <c r="G260" s="5"/>
-      <c r="H260" s="12"/>
-      <c r="I260" s="13"/>
-      <c r="J260" s="13"/>
-    </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="261" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A261" s="5"/>
       <c r="B261" s="5"/>
       <c r="C261" s="5"/>
@@ -3811,11 +3414,8 @@
       <c r="E261" s="5"/>
       <c r="F261" s="5"/>
       <c r="G261" s="5"/>
-      <c r="H261" s="12"/>
-      <c r="I261" s="13"/>
-      <c r="J261" s="13"/>
-    </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="262" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A262" s="5"/>
       <c r="B262" s="5"/>
       <c r="C262" s="5"/>
@@ -3823,11 +3423,8 @@
       <c r="E262" s="5"/>
       <c r="F262" s="5"/>
       <c r="G262" s="5"/>
-      <c r="H262" s="12"/>
-      <c r="I262" s="13"/>
-      <c r="J262" s="13"/>
-    </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="263" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A263" s="5"/>
       <c r="B263" s="5"/>
       <c r="C263" s="5"/>
@@ -3835,11 +3432,8 @@
       <c r="E263" s="5"/>
       <c r="F263" s="5"/>
       <c r="G263" s="5"/>
-      <c r="H263" s="12"/>
-      <c r="I263" s="13"/>
-      <c r="J263" s="13"/>
-    </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="264" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A264" s="5"/>
       <c r="B264" s="5"/>
       <c r="C264" s="5"/>
@@ -3847,11 +3441,8 @@
       <c r="E264" s="5"/>
       <c r="F264" s="5"/>
       <c r="G264" s="5"/>
-      <c r="H264" s="12"/>
-      <c r="I264" s="13"/>
-      <c r="J264" s="13"/>
-    </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="265" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A265" s="5"/>
       <c r="B265" s="5"/>
       <c r="C265" s="5"/>
@@ -3859,11 +3450,8 @@
       <c r="E265" s="5"/>
       <c r="F265" s="5"/>
       <c r="G265" s="5"/>
-      <c r="H265" s="12"/>
-      <c r="I265" s="13"/>
-      <c r="J265" s="13"/>
-    </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="266" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A266" s="5"/>
       <c r="B266" s="5"/>
       <c r="C266" s="5"/>
@@ -3871,11 +3459,8 @@
       <c r="E266" s="5"/>
       <c r="F266" s="5"/>
       <c r="G266" s="5"/>
-      <c r="H266" s="12"/>
-      <c r="I266" s="13"/>
-      <c r="J266" s="13"/>
-    </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A267" s="5"/>
       <c r="B267" s="5"/>
       <c r="C267" s="5"/>
@@ -3883,11 +3468,8 @@
       <c r="E267" s="5"/>
       <c r="F267" s="5"/>
       <c r="G267" s="5"/>
-      <c r="H267" s="12"/>
-      <c r="I267" s="13"/>
-      <c r="J267" s="13"/>
-    </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A268" s="5"/>
       <c r="B268" s="5"/>
       <c r="C268" s="5"/>
@@ -3895,11 +3477,8 @@
       <c r="E268" s="5"/>
       <c r="F268" s="5"/>
       <c r="G268" s="5"/>
-      <c r="H268" s="12"/>
-      <c r="I268" s="13"/>
-      <c r="J268" s="13"/>
-    </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="269" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A269" s="5"/>
       <c r="B269" s="5"/>
       <c r="C269" s="5"/>
@@ -3907,11 +3486,8 @@
       <c r="E269" s="5"/>
       <c r="F269" s="5"/>
       <c r="G269" s="5"/>
-      <c r="H269" s="12"/>
-      <c r="I269" s="13"/>
-      <c r="J269" s="13"/>
-    </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="270" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A270" s="5"/>
       <c r="B270" s="5"/>
       <c r="C270" s="5"/>
@@ -3919,11 +3495,8 @@
       <c r="E270" s="5"/>
       <c r="F270" s="5"/>
       <c r="G270" s="5"/>
-      <c r="H270" s="12"/>
-      <c r="I270" s="13"/>
-      <c r="J270" s="13"/>
-    </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="271" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A271" s="5"/>
       <c r="B271" s="5"/>
       <c r="C271" s="5"/>
@@ -3931,11 +3504,8 @@
       <c r="E271" s="5"/>
       <c r="F271" s="5"/>
       <c r="G271" s="5"/>
-      <c r="H271" s="12"/>
-      <c r="I271" s="13"/>
-      <c r="J271" s="13"/>
-    </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="272" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A272" s="5"/>
       <c r="B272" s="5"/>
       <c r="C272" s="5"/>
@@ -3943,11 +3513,8 @@
       <c r="E272" s="5"/>
       <c r="F272" s="5"/>
       <c r="G272" s="5"/>
-      <c r="H272" s="12"/>
-      <c r="I272" s="13"/>
-      <c r="J272" s="13"/>
-    </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="273" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A273" s="5"/>
       <c r="B273" s="5"/>
       <c r="C273" s="5"/>
@@ -3955,11 +3522,8 @@
       <c r="E273" s="5"/>
       <c r="F273" s="5"/>
       <c r="G273" s="5"/>
-      <c r="H273" s="12"/>
-      <c r="I273" s="13"/>
-      <c r="J273" s="13"/>
-    </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A274" s="5"/>
       <c r="B274" s="5"/>
       <c r="C274" s="5"/>
@@ -3967,11 +3531,8 @@
       <c r="E274" s="5"/>
       <c r="F274" s="5"/>
       <c r="G274" s="5"/>
-      <c r="H274" s="12"/>
-      <c r="I274" s="13"/>
-      <c r="J274" s="13"/>
-    </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A275" s="5"/>
       <c r="B275" s="5"/>
       <c r="C275" s="5"/>
@@ -3979,11 +3540,8 @@
       <c r="E275" s="5"/>
       <c r="F275" s="5"/>
       <c r="G275" s="5"/>
-      <c r="H275" s="12"/>
-      <c r="I275" s="13"/>
-      <c r="J275" s="13"/>
-    </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="276" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A276" s="5"/>
       <c r="B276" s="5"/>
       <c r="C276" s="5"/>
@@ -3991,11 +3549,8 @@
       <c r="E276" s="5"/>
       <c r="F276" s="5"/>
       <c r="G276" s="5"/>
-      <c r="H276" s="12"/>
-      <c r="I276" s="13"/>
-      <c r="J276" s="13"/>
-    </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="277" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A277" s="5"/>
       <c r="B277" s="5"/>
       <c r="C277" s="5"/>
@@ -4003,11 +3558,8 @@
       <c r="E277" s="5"/>
       <c r="F277" s="5"/>
       <c r="G277" s="5"/>
-      <c r="H277" s="12"/>
-      <c r="I277" s="13"/>
-      <c r="J277" s="13"/>
-    </row>
-    <row r="278" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A278" s="5"/>
       <c r="B278" s="5"/>
       <c r="C278" s="5"/>
@@ -4015,11 +3567,8 @@
       <c r="E278" s="5"/>
       <c r="F278" s="5"/>
       <c r="G278" s="5"/>
-      <c r="H278" s="12"/>
-      <c r="I278" s="13"/>
-      <c r="J278" s="13"/>
-    </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A279" s="5"/>
       <c r="B279" s="5"/>
       <c r="C279" s="5"/>
@@ -4027,11 +3576,8 @@
       <c r="E279" s="5"/>
       <c r="F279" s="5"/>
       <c r="G279" s="5"/>
-      <c r="H279" s="12"/>
-      <c r="I279" s="13"/>
-      <c r="J279" s="13"/>
-    </row>
-    <row r="280" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="280" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A280" s="5"/>
       <c r="B280" s="5"/>
       <c r="C280" s="5"/>
@@ -4039,11 +3585,8 @@
       <c r="E280" s="5"/>
       <c r="F280" s="5"/>
       <c r="G280" s="5"/>
-      <c r="H280" s="12"/>
-      <c r="I280" s="13"/>
-      <c r="J280" s="13"/>
-    </row>
-    <row r="281" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A281" s="5"/>
       <c r="B281" s="5"/>
       <c r="C281" s="5"/>
@@ -4051,11 +3594,8 @@
       <c r="E281" s="5"/>
       <c r="F281" s="5"/>
       <c r="G281" s="5"/>
-      <c r="H281" s="12"/>
-      <c r="I281" s="13"/>
-      <c r="J281" s="13"/>
-    </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A282" s="5"/>
       <c r="B282" s="5"/>
       <c r="C282" s="5"/>
@@ -4063,11 +3603,8 @@
       <c r="E282" s="5"/>
       <c r="F282" s="5"/>
       <c r="G282" s="5"/>
-      <c r="H282" s="12"/>
-      <c r="I282" s="13"/>
-      <c r="J282" s="13"/>
-    </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="283" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A283" s="5"/>
       <c r="B283" s="5"/>
       <c r="C283" s="5"/>
@@ -4075,11 +3612,8 @@
       <c r="E283" s="5"/>
       <c r="F283" s="5"/>
       <c r="G283" s="5"/>
-      <c r="H283" s="12"/>
-      <c r="I283" s="13"/>
-      <c r="J283" s="13"/>
-    </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="284" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A284" s="5"/>
       <c r="B284" s="5"/>
       <c r="C284" s="5"/>
@@ -4087,11 +3621,8 @@
       <c r="E284" s="5"/>
       <c r="F284" s="5"/>
       <c r="G284" s="5"/>
-      <c r="H284" s="12"/>
-      <c r="I284" s="13"/>
-      <c r="J284" s="13"/>
-    </row>
-    <row r="285" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A285" s="5"/>
       <c r="B285" s="5"/>
       <c r="C285" s="5"/>
@@ -4099,11 +3630,8 @@
       <c r="E285" s="5"/>
       <c r="F285" s="5"/>
       <c r="G285" s="5"/>
-      <c r="H285" s="12"/>
-      <c r="I285" s="13"/>
-      <c r="J285" s="13"/>
-    </row>
-    <row r="286" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="286" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A286" s="5"/>
       <c r="B286" s="5"/>
       <c r="C286" s="5"/>
@@ -4111,11 +3639,8 @@
       <c r="E286" s="5"/>
       <c r="F286" s="5"/>
       <c r="G286" s="5"/>
-      <c r="H286" s="12"/>
-      <c r="I286" s="13"/>
-      <c r="J286" s="13"/>
-    </row>
-    <row r="287" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="287" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A287" s="5"/>
       <c r="B287" s="5"/>
       <c r="C287" s="5"/>
@@ -4123,11 +3648,8 @@
       <c r="E287" s="5"/>
       <c r="F287" s="5"/>
       <c r="G287" s="5"/>
-      <c r="H287" s="12"/>
-      <c r="I287" s="13"/>
-      <c r="J287" s="13"/>
-    </row>
-    <row r="288" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A288" s="5"/>
       <c r="B288" s="5"/>
       <c r="C288" s="5"/>
@@ -4135,11 +3657,8 @@
       <c r="E288" s="5"/>
       <c r="F288" s="5"/>
       <c r="G288" s="5"/>
-      <c r="H288" s="12"/>
-      <c r="I288" s="13"/>
-      <c r="J288" s="13"/>
-    </row>
-    <row r="289" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="289" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A289" s="5"/>
       <c r="B289" s="5"/>
       <c r="C289" s="5"/>
@@ -4147,11 +3666,8 @@
       <c r="E289" s="5"/>
       <c r="F289" s="5"/>
       <c r="G289" s="5"/>
-      <c r="H289" s="12"/>
-      <c r="I289" s="13"/>
-      <c r="J289" s="13"/>
-    </row>
-    <row r="290" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="290" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A290" s="5"/>
       <c r="B290" s="5"/>
       <c r="C290" s="5"/>
@@ -4159,11 +3675,8 @@
       <c r="E290" s="5"/>
       <c r="F290" s="5"/>
       <c r="G290" s="5"/>
-      <c r="H290" s="12"/>
-      <c r="I290" s="13"/>
-      <c r="J290" s="13"/>
-    </row>
-    <row r="291" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="291" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A291" s="5"/>
       <c r="B291" s="5"/>
       <c r="C291" s="5"/>
@@ -4171,11 +3684,8 @@
       <c r="E291" s="5"/>
       <c r="F291" s="5"/>
       <c r="G291" s="5"/>
-      <c r="H291" s="12"/>
-      <c r="I291" s="13"/>
-      <c r="J291" s="13"/>
-    </row>
-    <row r="292" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="292" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A292" s="5"/>
       <c r="B292" s="5"/>
       <c r="C292" s="5"/>
@@ -4183,11 +3693,8 @@
       <c r="E292" s="5"/>
       <c r="F292" s="5"/>
       <c r="G292" s="5"/>
-      <c r="H292" s="12"/>
-      <c r="I292" s="13"/>
-      <c r="J292" s="13"/>
-    </row>
-    <row r="293" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="293" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A293" s="5"/>
       <c r="B293" s="5"/>
       <c r="C293" s="5"/>
@@ -4195,11 +3702,8 @@
       <c r="E293" s="5"/>
       <c r="F293" s="5"/>
       <c r="G293" s="5"/>
-      <c r="H293" s="12"/>
-      <c r="I293" s="13"/>
-      <c r="J293" s="13"/>
-    </row>
-    <row r="294" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="294" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A294" s="5"/>
       <c r="B294" s="5"/>
       <c r="C294" s="5"/>
@@ -4207,11 +3711,8 @@
       <c r="E294" s="5"/>
       <c r="F294" s="5"/>
       <c r="G294" s="5"/>
-      <c r="H294" s="12"/>
-      <c r="I294" s="13"/>
-      <c r="J294" s="13"/>
-    </row>
-    <row r="295" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="295" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A295" s="5"/>
       <c r="B295" s="5"/>
       <c r="C295" s="5"/>
@@ -4219,11 +3720,8 @@
       <c r="E295" s="5"/>
       <c r="F295" s="5"/>
       <c r="G295" s="5"/>
-      <c r="H295" s="12"/>
-      <c r="I295" s="13"/>
-      <c r="J295" s="13"/>
-    </row>
-    <row r="296" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="296" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A296" s="5"/>
       <c r="B296" s="5"/>
       <c r="C296" s="5"/>
@@ -4231,11 +3729,8 @@
       <c r="E296" s="5"/>
       <c r="F296" s="5"/>
       <c r="G296" s="5"/>
-      <c r="H296" s="12"/>
-      <c r="I296" s="13"/>
-      <c r="J296" s="13"/>
-    </row>
-    <row r="297" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="297" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A297" s="5"/>
       <c r="B297" s="5"/>
       <c r="C297" s="5"/>
@@ -4243,11 +3738,8 @@
       <c r="E297" s="5"/>
       <c r="F297" s="5"/>
       <c r="G297" s="5"/>
-      <c r="H297" s="12"/>
-      <c r="I297" s="13"/>
-      <c r="J297" s="13"/>
-    </row>
-    <row r="298" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="298" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A298" s="5"/>
       <c r="B298" s="5"/>
       <c r="C298" s="5"/>
@@ -4255,11 +3747,8 @@
       <c r="E298" s="5"/>
       <c r="F298" s="5"/>
       <c r="G298" s="5"/>
-      <c r="H298" s="12"/>
-      <c r="I298" s="13"/>
-      <c r="J298" s="13"/>
-    </row>
-    <row r="299" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="299" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A299" s="5"/>
       <c r="B299" s="5"/>
       <c r="C299" s="5"/>
@@ -4267,11 +3756,8 @@
       <c r="E299" s="5"/>
       <c r="F299" s="5"/>
       <c r="G299" s="5"/>
-      <c r="H299" s="12"/>
-      <c r="I299" s="13"/>
-      <c r="J299" s="13"/>
-    </row>
-    <row r="300" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A300" s="5"/>
       <c r="B300" s="5"/>
       <c r="C300" s="5"/>
@@ -4279,11 +3765,8 @@
       <c r="E300" s="5"/>
       <c r="F300" s="5"/>
       <c r="G300" s="5"/>
-      <c r="H300" s="12"/>
-      <c r="I300" s="13"/>
-      <c r="J300" s="13"/>
-    </row>
-    <row r="301" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A301" s="5"/>
       <c r="B301" s="5"/>
       <c r="C301" s="5"/>
@@ -4291,13 +3774,10 @@
       <c r="E301" s="5"/>
       <c r="F301" s="5"/>
       <c r="G301" s="5"/>
-      <c r="H301" s="12"/>
-      <c r="I301" s="13"/>
-      <c r="J301" s="13"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J20" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Get policy from Excel
</commit_message>
<xml_diff>
--- a/pages/UATStability.xlsx
+++ b/pages/UATStability.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA83F1AE-295A-4EA7-B299-D4D71371E704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21484C32-1155-49EC-999E-13596D1BA352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$18</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -564,7 +564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:J299"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.453125" style="4" customWidth="1"/>
@@ -707,7 +707,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -777,7 +777,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="7"/>
-      <c r="B9" s="10"/>
+      <c r="B9" s="6"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
@@ -789,7 +789,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="7"/>
-      <c r="B10" s="10"/>
+      <c r="B10" s="6"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
@@ -885,7 +885,7 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="7"/>
-      <c r="B18" s="6"/>
+      <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
@@ -896,8 +896,8 @@
       <c r="J18" s="9"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="7"/>
-      <c r="B19" s="6"/>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
@@ -908,7 +908,7 @@
       <c r="J19" s="9"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="7"/>
+      <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
@@ -1384,8 +1384,8 @@
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
       <c r="H59" s="5"/>
-      <c r="I59" s="9"/>
-      <c r="J59" s="9"/>
+      <c r="I59" s="13"/>
+      <c r="J59" s="13"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5"/>
@@ -1396,8 +1396,8 @@
       <c r="F60" s="5"/>
       <c r="G60" s="5"/>
       <c r="H60" s="5"/>
-      <c r="I60" s="9"/>
-      <c r="J60" s="9"/>
+      <c r="I60" s="13"/>
+      <c r="J60" s="13"/>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5"/>
@@ -2209,13 +2209,10 @@
       <c r="C128" s="5"/>
       <c r="D128" s="5"/>
       <c r="E128" s="5"/>
-      <c r="F128" s="5"/>
-      <c r="G128" s="5"/>
-      <c r="H128" s="5"/>
-      <c r="I128" s="13"/>
-      <c r="J128" s="13"/>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F128" s="12"/>
+      <c r="G128" s="12"/>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129" s="5"/>
       <c r="B129" s="5"/>
       <c r="C129" s="5"/>
@@ -2223,20 +2220,17 @@
       <c r="E129" s="5"/>
       <c r="F129" s="5"/>
       <c r="G129" s="5"/>
-      <c r="H129" s="5"/>
-      <c r="I129" s="13"/>
-      <c r="J129" s="13"/>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" s="5"/>
       <c r="B130" s="5"/>
       <c r="C130" s="5"/>
       <c r="D130" s="5"/>
       <c r="E130" s="5"/>
-      <c r="F130" s="12"/>
-      <c r="G130" s="12"/>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F130" s="5"/>
+      <c r="G130" s="5"/>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" s="5"/>
       <c r="B131" s="5"/>
       <c r="C131" s="5"/>
@@ -2245,7 +2239,7 @@
       <c r="F131" s="5"/>
       <c r="G131" s="5"/>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" s="5"/>
       <c r="B132" s="5"/>
       <c r="C132" s="5"/>
@@ -2254,7 +2248,7 @@
       <c r="F132" s="5"/>
       <c r="G132" s="5"/>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133" s="5"/>
       <c r="B133" s="5"/>
       <c r="C133" s="5"/>
@@ -2263,7 +2257,7 @@
       <c r="F133" s="5"/>
       <c r="G133" s="5"/>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134" s="5"/>
       <c r="B134" s="5"/>
       <c r="C134" s="5"/>
@@ -2272,7 +2266,7 @@
       <c r="F134" s="5"/>
       <c r="G134" s="5"/>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135" s="5"/>
       <c r="B135" s="5"/>
       <c r="C135" s="5"/>
@@ -2281,7 +2275,7 @@
       <c r="F135" s="5"/>
       <c r="G135" s="5"/>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" s="5"/>
       <c r="B136" s="5"/>
       <c r="C136" s="5"/>
@@ -2290,7 +2284,7 @@
       <c r="F136" s="5"/>
       <c r="G136" s="5"/>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" s="5"/>
       <c r="B137" s="5"/>
       <c r="C137" s="5"/>
@@ -2299,7 +2293,7 @@
       <c r="F137" s="5"/>
       <c r="G137" s="5"/>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" s="5"/>
       <c r="B138" s="5"/>
       <c r="C138" s="5"/>
@@ -2308,7 +2302,7 @@
       <c r="F138" s="5"/>
       <c r="G138" s="5"/>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139" s="5"/>
       <c r="B139" s="5"/>
       <c r="C139" s="5"/>
@@ -2317,7 +2311,7 @@
       <c r="F139" s="5"/>
       <c r="G139" s="5"/>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140" s="5"/>
       <c r="B140" s="5"/>
       <c r="C140" s="5"/>
@@ -2326,7 +2320,7 @@
       <c r="F140" s="5"/>
       <c r="G140" s="5"/>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141" s="5"/>
       <c r="B141" s="5"/>
       <c r="C141" s="5"/>
@@ -2335,7 +2329,7 @@
       <c r="F141" s="5"/>
       <c r="G141" s="5"/>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142" s="5"/>
       <c r="B142" s="5"/>
       <c r="C142" s="5"/>
@@ -2344,7 +2338,7 @@
       <c r="F142" s="5"/>
       <c r="G142" s="5"/>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" s="5"/>
       <c r="B143" s="5"/>
       <c r="C143" s="5"/>
@@ -2353,7 +2347,7 @@
       <c r="F143" s="5"/>
       <c r="G143" s="5"/>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144" s="5"/>
       <c r="B144" s="5"/>
       <c r="C144" s="5"/>
@@ -3757,27 +3751,9 @@
       <c r="F299" s="5"/>
       <c r="G299" s="5"/>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A300" s="5"/>
-      <c r="B300" s="5"/>
-      <c r="C300" s="5"/>
-      <c r="D300" s="5"/>
-      <c r="E300" s="5"/>
-      <c r="F300" s="5"/>
-      <c r="G300" s="5"/>
-    </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A301" s="5"/>
-      <c r="B301" s="5"/>
-      <c r="C301" s="5"/>
-      <c r="D301" s="5"/>
-      <c r="E301" s="5"/>
-      <c r="F301" s="5"/>
-      <c r="G301" s="5"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J20" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:J18" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
PA and Motor endorsement updated
</commit_message>
<xml_diff>
--- a/pages/UATStability.xlsx
+++ b/pages/UATStability.xlsx
@@ -958,7 +958,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="5" t="n">
         <v>8</v>
       </c>
@@ -1010,29 +1010,109 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="n"/>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>RV</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Third Party</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>1000068384</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>00000402000070380</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>25-05-2026</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Downloaded Automatically
+Validated Manually</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Downloaded Automatically
+Validated Manually</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="6" t="n"/>
-      <c r="J11" s="6" t="n"/>
+      <c r="A11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Personal Accident Safe</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>1000068444</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>00000402000070405</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>25-05-2026</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>Downloaded Automatically
+Validated Manually</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Downloaded Automatically
+Validated Manually</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>

</xml_diff>